<commit_message>
Calibrate input.xlsx with verified real-life market data from BYMA, BCRA, Rava, Ecovalores, and Matba Rofex
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -450,7 +450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -461,6 +461,7 @@
     <col width="35" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -504,6 +505,11 @@
           <t>Beta</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Price_ARS_BYMA</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -517,10 +523,10 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>25000</v>
+        <v>151257</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>32</v>
+        <v>5.289</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>800000</v>
@@ -538,6 +544,9 @@
       <c r="H2" s="2" t="n">
         <v>1.05</v>
       </c>
+      <c r="I2" s="2" t="n">
+        <v>8370</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -551,10 +560,10 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>160000</v>
+        <v>181900</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>5</v>
+        <v>4.398</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>800000</v>
@@ -572,6 +581,9 @@
       <c r="H3" s="2" t="n">
         <v>1.18</v>
       </c>
+      <c r="I3" s="2" t="n">
+        <v>6960</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -585,10 +597,10 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>80000</v>
+        <v>149031</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>6.25</v>
+        <v>3.355</v>
       </c>
       <c r="E4" s="2" t="n">
         <v>500000</v>
@@ -606,6 +618,9 @@
       <c r="H4" s="2" t="n">
         <v>0.95</v>
       </c>
+      <c r="I4" s="2" t="n">
+        <v>5310</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -619,10 +634,10 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>70000</v>
+        <v>63922</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>7.142857</v>
+        <v>7.822</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>500000</v>
@@ -640,6 +655,9 @@
       <c r="H5" s="2" t="n">
         <v>1.15</v>
       </c>
+      <c r="I5" s="2" t="n">
+        <v>12380</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -653,10 +671,10 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>400000</v>
+        <v>909504</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>1</v>
+        <v>0.4398</v>
       </c>
       <c r="E6" s="2" t="n">
         <v>400000</v>
@@ -666,9 +684,16 @@
           <t>Materials / Steel &amp; Industrial</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr"/>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
       <c r="H6" s="2" t="n">
         <v>0.88</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>696</v>
       </c>
     </row>
   </sheetData>
@@ -784,10 +809,10 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>1935484</v>
+        <v>2068966</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>0.62</v>
+        <v>0.58</v>
       </c>
       <c r="F2" s="2" t="n">
         <v>1200000</v>
@@ -798,22 +823,22 @@
         </is>
       </c>
       <c r="H2" s="2" t="n">
-        <v>4.5</v>
+        <v>3.8</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>0.0075</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>0.165</v>
+        <v>0.0634</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>2.63</v>
+        <v>2.52</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>8.92</v>
+        <v>8.5</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>315.6</v>
+        <v>300</v>
       </c>
     </row>
     <row r="3">
@@ -833,10 +858,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>2068965</v>
+        <v>2145923</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>0.58</v>
+        <v>0.5592</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>1200000</v>
@@ -847,22 +872,22 @@
         </is>
       </c>
       <c r="H3" s="2" t="n">
-        <v>4.5</v>
+        <v>3.8</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>0.0075</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>0.182</v>
+        <v>0.0725</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>2.56</v>
+        <v>2.45</v>
       </c>
       <c r="L3" s="2" t="n">
-        <v>8.5</v>
+        <v>8.1</v>
       </c>
       <c r="M3" s="2" t="n">
-        <v>307.2</v>
+        <v>290</v>
       </c>
     </row>
     <row r="4">
@@ -882,10 +907,10 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>2040816</v>
+        <v>1248284</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0.49</v>
+        <v>0.8011</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>1000000</v>
@@ -896,22 +921,22 @@
         </is>
       </c>
       <c r="H4" s="2" t="n">
-        <v>9.5</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="I4" s="2" t="n">
         <v>0.03625</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>0.158</v>
+        <v>0.093</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>4.98</v>
+        <v>4.68</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>34.1</v>
+        <v>28.5</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>498</v>
+        <v>460</v>
       </c>
     </row>
     <row r="5">
@@ -931,10 +956,10 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>1739130</v>
+        <v>1039231</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>0.46</v>
+        <v>0.7698</v>
       </c>
       <c r="F5" s="2" t="n">
         <v>800000</v>
@@ -945,22 +970,22 @@
         </is>
       </c>
       <c r="H5" s="2" t="n">
-        <v>9.5</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="I5" s="2" t="n">
         <v>0.03625</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>0.171</v>
+        <v>0.102</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>4.82</v>
+        <v>4.55</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>32.5</v>
+        <v>26.8</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>385.6</v>
+        <v>360</v>
       </c>
     </row>
     <row r="6">
@@ -980,10 +1005,10 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>1509434</v>
+        <v>948992</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>0.53</v>
+        <v>0.843</v>
       </c>
       <c r="F6" s="2" t="n">
         <v>800000</v>
@@ -994,22 +1019,22 @@
         </is>
       </c>
       <c r="H6" s="2" t="n">
-        <v>12</v>
+        <v>11.3</v>
       </c>
       <c r="I6" s="2" t="n">
         <v>0.0425</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>0.152</v>
+        <v>0.0897</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>5.58</v>
+        <v>5.3</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>44.8</v>
+        <v>38.2</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>446.4</v>
+        <v>420</v>
       </c>
     </row>
   </sheetData>
@@ -1039,7 +1064,7 @@
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="52" customWidth="1" min="14" max="14"/>
+    <col width="79" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1164,7 +1189,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>Long USD hedge contract against ARS depreciation</t>
+          <t>Rofex Nov 2026 contract @ 1,580.50 ARS. 1.0 delta hedge against devaluation</t>
         </is>
       </c>
     </row>
@@ -1185,10 +1210,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1600</v>
+        <v>1819</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>262.5</v>
+        <v>230.9</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>420000</v>
@@ -1205,20 +1230,20 @@
         <v>0.54</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>0.082</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>980</v>
+        <v>920</v>
       </c>
       <c r="L3" s="2" t="n">
-        <v>-1250</v>
+        <v>-1180</v>
       </c>
       <c r="M3" s="2" t="n">
         <v>0</v>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>Call Option ATM 45 days strike $5.00</t>
+          <t>Call Option ATM 45D strike $4.42 USD ($7,000 ARS). IV: 62%</t>
         </is>
       </c>
     </row>
@@ -1239,10 +1264,10 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>1600</v>
+        <v>1819</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>175</v>
+        <v>153.93</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>280000</v>
@@ -1259,20 +1284,20 @@
         <v>-0.28</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>0.065</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>720</v>
+        <v>680</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>-920</v>
+        <v>-850</v>
       </c>
       <c r="M4" s="2" t="n">
         <v>0</v>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>Protective Put OTM strike $4.50</t>
+          <t>Protective Put OTM strike $3.98 USD ($6,300 ARS). IV: 68%</t>
         </is>
       </c>
     </row>
@@ -1326,7 +1351,7 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>Synthetic long USD / short ARS forward</t>
+          <t>OTC NDF forward contract @ 1,638 ARS synthetic long USD</t>
         </is>
       </c>
     </row>
@@ -1380,7 +1405,7 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>Pay Fixed 40% / Receive Floating BADLAR</t>
+          <t>Pay Fixed 24.0% ARS / Receive Floating BADLAR 23.25% + 150 bps</t>
         </is>
       </c>
     </row>
@@ -1395,7 +1420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -1444,86 +1469,131 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>1280</v>
+        <v>1582.6</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>CCL exchange rate for USD/ARS conversion</t>
+          <t>Contado con Liquidacion (CCL) market exchange rate</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Default_Confidence_Level</t>
+          <t>USD_ARS_MEP_Rate</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>0.95</v>
+        <v>1526.9</v>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Baseline VaR confidence interval (e.g. 0.95, 0.99)</t>
+          <t>Dólar Bolsa (MEP) market exchange rate</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Default_Holding_Period_Days</t>
+          <t>USD_ARS_Mayorista_Rate</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>1</v>
+        <v>1508</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Holding period horizon in trading days</t>
+          <t>Official Wholesale exchange rate (BCRA)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Stress_Vol_Multiplier</t>
+          <t>BADLAR_TNA_Percent</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>2.2</v>
+        <v>23.25</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Volatility scaling factor under stressed regime</t>
+          <t>BCRA BADLAR benchmark rate for private banks</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Stress_Correlation_Spike</t>
+          <t>Default_Confidence_Level</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>0.9</v>
+        <v>0.95</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Correlation convergence level during market stress</t>
+          <t>Baseline VaR confidence interval (e.g. 0.95, 0.99)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
+          <t>Default_Holding_Period_Days</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Holding period horizon in trading days</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Stress_Vol_Multiplier</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Volatility scaling factor under stressed regime</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Stress_Correlation_Spike</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Correlation convergence level during market stress</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
           <t>Reporting_Month</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>September 2026</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Monthly reporting cycle label</t>
         </is>

</xml_diff>

<commit_message>
Add retail investor mode, cash/liquidity class, Cocos broker CSV loader, and monthly executive briefing
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -10,7 +10,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bonds" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Derivatives" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash_Liquidity" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1420,6 +1421,128 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="43" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="53" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Amount_USD</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Amount_ARS</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Annual_Yield_Pct</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>CAUCION_ARS</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Caución Bursátil 7D (BYMA)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Caución Bursátil</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>300000</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>474780000</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Short term 7-day repo backed by sovereign bonds</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>CASH_USD</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Dólares Disponibles en Cuenta (MEP/CCL)</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Liquid Cash USD</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>200000</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>316520000</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Liquid USD cash reserves for opportunistic buying</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>